<commit_message>
sync: sessao de 05-06/08 — travessia verde, whatsapp com botoes, google pronto
Sistema: login com Google montado e provado (13/13, so falta o client_id do
console), modelo de WhatsApp com botoes aprovado e ativo, rodape unico dos
emails com o telefone real, webhook aceitando www e barra final, apagarConta
limpando o acervo R2 (6 orfaos de teste apagados do bucket).

Comercial: proposta em PDF numa folha (24/24), suporte na proposta desde o
inicio, faturar.py com teto proporcional do MEI e parcelas a receber (56/56),
clientes-atendidos.json limpo e versionado, prospeccao e suporte escritos.

Padroes: memorial com 33 campos respondidos, base de dissipacao semeada de
catalogo com fonte citada, marcador de logo do cliente em 4 formatos.

Marca: logo realinhado pela tinta (fio acompanha o nome), PNGs refeitos com
a Inter.

Travessia ponta a ponta contra producao: 41/41. Bateria completa: 141/141.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/padroes/templates/xlsx/MODELO - Design Térmico.xlsx
+++ b/padroes/templates/xlsx/MODELO - Design Térmico.xlsx
@@ -848,7 +848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -858,7 +858,7 @@
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -911,27 +911,466 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr"/>
-      <c r="B4" s="4" t="inlineStr"/>
-      <c r="C4" s="7" t="inlineStr"/>
-      <c r="D4" s="7" t="inlineStr"/>
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Disjuntor</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>MDWH</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Minidisjuntor In &lt; 10 A — por polo</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>WEG</t>
+        </is>
+      </c>
       <c r="E4" s="4" t="inlineStr"/>
-      <c r="F4" s="4" t="inlineStr"/>
-      <c r="G4" s="4">
-        <f>E4+F4</f>
+      <c r="F4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>WEG MDW 50163906 p.17 (05/08/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Disjuntor</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>MDWH</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Minidisjuntor 10 a 16 A — por polo</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>WEG</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr"/>
+      <c r="F5" s="4" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>WEG MDW 50163906 p.17 (05/08/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Disjuntor</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>MDWH</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Minidisjuntor 16 a 25 A — por polo</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>WEG</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr"/>
+      <c r="F6" s="4" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>WEG MDW 50163906 p.17 (05/08/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Disjuntor</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>MDWH</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Minidisjuntor 25 a 32 A — por polo</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>WEG</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr"/>
+      <c r="F7" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>WEG MDW 50163906 p.17 (05/08/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Disjuntor</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>MDWH</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Minidisjuntor 32 a 40 A — por polo</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>WEG</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr"/>
+      <c r="F8" s="4" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>WEG MDW 50163906 p.17 (05/08/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Disjuntor</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>MDWH</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Minidisjuntor 40 a 50 A — por polo</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>WEG</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr"/>
+      <c r="F9" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>WEG MDW 50163906 p.17 (05/08/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Disjuntor</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>MDWH</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Minidisjuntor 50 a 63 A — por polo</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>WEG</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr"/>
+      <c r="F10" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>WEG MDW 50163906 p.17 (05/08/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Disjuntor</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>MDWH</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Minidisjuntor 63 a 100 A — por polo</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>WEG</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr"/>
+      <c r="F11" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>WEG MDW 50163906 p.17 (05/08/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Disjuntor</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>MDWH</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Minidisjuntor 100 a 125 A — por polo</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>WEG</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr"/>
+      <c r="F12" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>WEG MDW 50163906 p.17 (05/08/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Contator</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>CWB</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Bobina CC, contator até 38 A (máximo)</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>WEG</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="F13" s="4" t="inlineStr"/>
+      <c r="G13" s="4" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>WEG CWB 50042424 p.7 (05/08/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Contator</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>CWB</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Bobina CA, contator até 38 A — 7,5 VA</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>WEG</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F14" s="4" t="inlineStr"/>
+      <c r="G14" s="4" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>WEG CWB 50042424 p.7 (05/08/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Fonte 24 VCC</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr"/>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>CALCULADO: Psaída x (1/rend - 1). Ex.: 240 W a 93% = 18 W</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr"/>
+      <c r="E15" s="4" t="inlineStr"/>
+      <c r="F15" s="4" t="inlineStr"/>
+      <c r="G15" s="4" t="inlineStr"/>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>rendimento do datasheet do modelo</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Inversor</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr"/>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>CALCULADO: Pmotor x (1 - rend). Ex.: 5,5 kW a 97% = 165 W</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr"/>
+      <c r="E16" s="4" t="inlineStr"/>
+      <c r="F16" s="4" t="inlineStr"/>
+      <c r="G16" s="4" t="inlineStr"/>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>rendimento do datasheet do modelo</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr"/>
+      <c r="B17" s="4" t="inlineStr"/>
+      <c r="C17" s="7" t="inlineStr"/>
+      <c r="D17" s="7" t="inlineStr"/>
+      <c r="E17" s="4" t="inlineStr"/>
+      <c r="F17" s="4" t="inlineStr"/>
+      <c r="G17" s="4">
+        <f>E17+F17</f>
         <v/>
       </c>
-      <c r="H4" s="7" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>Preencher a partir do catálogo de cada fabricante. Esta base cresce a cada projeto e é ativo próprio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="H17" s="7" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>As linhas acima vieram do catálogo do fabricante, com documento e data na última coluna. Conferir na revisão do catálogo em uso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>Disjuntor: o valor é POR POLO — multiplicar pelo número de polos. E é o MÁXIMO da norma, não o típico medido: erra a favor do frio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>Fonte e inversor não têm valor de tabela: a dissipação sai do rendimento. Ver as duas últimas linhas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>Esta base cresce a cada projeto e é ativo próprio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>Nunca copiar base de dados de terceiros — o dado é público no datasheet, a compilação é sua.</t>
         </is>

</xml_diff>